<commit_message>
planilha atualizada (105037 bytes) + rebuild data.js
</commit_message>
<xml_diff>
--- a/Mapa - Zelar.xlsx
+++ b/Mapa - Zelar.xlsx
@@ -15240,7 +15240,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" hidden="1">
       <c r="A2" t="s">
         <v>17</v>
       </c>
@@ -15293,7 +15293,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" hidden="1">
       <c r="A3" t="s">
         <v>31</v>
       </c>
@@ -15346,7 +15346,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" hidden="1">
       <c r="A4" t="s">
         <v>43</v>
       </c>
@@ -15399,7 +15399,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" hidden="1">
       <c r="A5" t="s">
         <v>52</v>
       </c>
@@ -15452,7 +15452,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" hidden="1">
       <c r="A6" t="s">
         <v>64</v>
       </c>
@@ -15505,7 +15505,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" hidden="1">
       <c r="A7" t="s">
         <v>52</v>
       </c>
@@ -15558,7 +15558,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" hidden="1">
       <c r="A8" t="s">
         <v>80</v>
       </c>
@@ -15611,7 +15611,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" hidden="1">
       <c r="A9" t="s">
         <v>91</v>
       </c>
@@ -15664,7 +15664,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" hidden="1">
       <c r="A10" t="s">
         <v>91</v>
       </c>
@@ -15717,7 +15717,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" hidden="1">
       <c r="A11" t="s">
         <v>91</v>
       </c>
@@ -15770,7 +15770,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" hidden="1">
       <c r="A12" t="s">
         <v>112</v>
       </c>
@@ -15814,7 +15814,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" hidden="1">
       <c r="A13" t="s">
         <v>119</v>
       </c>
@@ -15867,7 +15867,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" hidden="1">
       <c r="A14" t="s">
         <v>119</v>
       </c>
@@ -15920,7 +15920,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" hidden="1">
       <c r="A15" t="s">
         <v>135</v>
       </c>
@@ -15973,7 +15973,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" hidden="1">
       <c r="A16" t="s">
         <v>146</v>
       </c>
@@ -16026,7 +16026,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" hidden="1">
       <c r="A17" t="s">
         <v>154</v>
       </c>
@@ -16079,7 +16079,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" hidden="1">
       <c r="A18" t="s">
         <v>161</v>
       </c>
@@ -16132,7 +16132,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" hidden="1">
       <c r="A19" t="s">
         <v>166</v>
       </c>
@@ -16185,7 +16185,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" hidden="1">
       <c r="A20" t="s">
         <v>171</v>
       </c>
@@ -16238,7 +16238,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" hidden="1">
       <c r="A21" t="s">
         <v>171</v>
       </c>
@@ -16291,7 +16291,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" hidden="1">
       <c r="A22" t="s">
         <v>171</v>
       </c>
@@ -16344,7 +16344,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" hidden="1">
       <c r="A23" t="s">
         <v>171</v>
       </c>
@@ -16397,7 +16397,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" hidden="1">
       <c r="A24" t="s">
         <v>193</v>
       </c>
@@ -16450,7 +16450,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" hidden="1">
       <c r="A25" t="s">
         <v>193</v>
       </c>
@@ -16503,7 +16503,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" hidden="1">
       <c r="A26" t="s">
         <v>193</v>
       </c>
@@ -16556,7 +16556,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" hidden="1">
       <c r="A27" t="s">
         <v>193</v>
       </c>
@@ -16609,7 +16609,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" hidden="1">
       <c r="A28" t="s">
         <v>213</v>
       </c>
@@ -16662,7 +16662,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" hidden="1">
       <c r="A29" t="s">
         <v>221</v>
       </c>
@@ -16715,7 +16715,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" hidden="1">
       <c r="A30" t="s">
         <v>231</v>
       </c>
@@ -16768,7 +16768,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" hidden="1">
       <c r="A31" t="s">
         <v>239</v>
       </c>
@@ -16821,7 +16821,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" hidden="1">
       <c r="A32" t="s">
         <v>239</v>
       </c>
@@ -16874,7 +16874,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" hidden="1">
       <c r="A33" t="s">
         <v>239</v>
       </c>
@@ -16927,7 +16927,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" hidden="1">
       <c r="A34" t="s">
         <v>263</v>
       </c>
@@ -16980,7 +16980,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" hidden="1">
       <c r="A35" t="s">
         <v>239</v>
       </c>
@@ -17033,7 +17033,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" hidden="1">
       <c r="A36" t="s">
         <v>279</v>
       </c>
@@ -17086,7 +17086,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" hidden="1">
       <c r="A37" t="s">
         <v>287</v>
       </c>
@@ -17139,7 +17139,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" hidden="1">
       <c r="A38" t="s">
         <v>291</v>
       </c>
@@ -17192,7 +17192,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" hidden="1">
       <c r="A39" t="s">
         <v>298</v>
       </c>
@@ -17245,7 +17245,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" hidden="1">
       <c r="A40" t="s">
         <v>298</v>
       </c>
@@ -17298,7 +17298,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" hidden="1">
       <c r="A41" t="s">
         <v>298</v>
       </c>
@@ -17351,7 +17351,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="42">
+    <row r="42" hidden="1">
       <c r="A42" t="s">
         <v>298</v>
       </c>
@@ -17404,7 +17404,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="43">
+    <row r="43" hidden="1">
       <c r="A43" t="s">
         <v>298</v>
       </c>
@@ -17457,7 +17457,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" hidden="1">
       <c r="A44" t="s">
         <v>298</v>
       </c>
@@ -17510,7 +17510,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" hidden="1">
       <c r="A45" t="s">
         <v>298</v>
       </c>
@@ -17563,7 +17563,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="46">
+    <row r="46" hidden="1">
       <c r="A46" t="s">
         <v>298</v>
       </c>
@@ -17616,7 +17616,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="47">
+    <row r="47" hidden="1">
       <c r="A47" t="s">
         <v>298</v>
       </c>
@@ -17669,7 +17669,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="48">
+    <row r="48" hidden="1">
       <c r="A48" t="s">
         <v>298</v>
       </c>
@@ -17722,7 +17722,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="49">
+    <row r="49" hidden="1">
       <c r="A49" t="s">
         <v>298</v>
       </c>
@@ -17775,7 +17775,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="50">
+    <row r="50" hidden="1">
       <c r="A50" t="s">
         <v>298</v>
       </c>
@@ -17828,7 +17828,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="51">
+    <row r="51" hidden="1">
       <c r="A51" t="s">
         <v>298</v>
       </c>
@@ -17881,7 +17881,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="52">
+    <row r="52" hidden="1">
       <c r="A52" t="s">
         <v>298</v>
       </c>
@@ -17934,7 +17934,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="53">
+    <row r="53" hidden="1">
       <c r="A53" t="s">
         <v>298</v>
       </c>
@@ -17987,7 +17987,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="54">
+    <row r="54" hidden="1">
       <c r="A54" t="s">
         <v>298</v>
       </c>
@@ -18040,7 +18040,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="55">
+    <row r="55" hidden="1">
       <c r="A55" t="s">
         <v>361</v>
       </c>
@@ -18093,7 +18093,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="56">
+    <row r="56" hidden="1">
       <c r="A56" t="s">
         <v>361</v>
       </c>
@@ -18146,7 +18146,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="57">
+    <row r="57" hidden="1">
       <c r="A57" t="s">
         <v>361</v>
       </c>
@@ -18199,7 +18199,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="58">
+    <row r="58" hidden="1">
       <c r="A58" t="s">
         <v>361</v>
       </c>
@@ -18252,7 +18252,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="59">
+    <row r="59" hidden="1">
       <c r="A59" t="s">
         <v>361</v>
       </c>
@@ -18305,7 +18305,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="60">
+    <row r="60" hidden="1">
       <c r="A60" t="s">
         <v>361</v>
       </c>
@@ -18358,7 +18358,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="61">
+    <row r="61" hidden="1">
       <c r="A61" t="s">
         <v>361</v>
       </c>
@@ -18411,7 +18411,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="62">
+    <row r="62" hidden="1">
       <c r="A62" t="s">
         <v>361</v>
       </c>
@@ -18464,7 +18464,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="63">
+    <row r="63" hidden="1">
       <c r="A63" t="s">
         <v>361</v>
       </c>
@@ -18517,7 +18517,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="64">
+    <row r="64" hidden="1">
       <c r="A64" t="s">
         <v>361</v>
       </c>
@@ -18570,7 +18570,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="65">
+    <row r="65" hidden="1">
       <c r="A65" t="s">
         <v>361</v>
       </c>
@@ -18623,7 +18623,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="66">
+    <row r="66" hidden="1">
       <c r="A66" t="s">
         <v>361</v>
       </c>
@@ -18676,7 +18676,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="67">
+    <row r="67" hidden="1">
       <c r="A67" t="s">
         <v>361</v>
       </c>
@@ -18729,7 +18729,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="68">
+    <row r="68" hidden="1">
       <c r="A68" t="s">
         <v>361</v>
       </c>
@@ -18782,7 +18782,7 @@
         <v>426</v>
       </c>
     </row>
-    <row r="69">
+    <row r="69" hidden="1">
       <c r="A69" t="s">
         <v>361</v>
       </c>
@@ -18835,7 +18835,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="70">
+    <row r="70" hidden="1">
       <c r="A70" t="s">
         <v>432</v>
       </c>
@@ -18888,7 +18888,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="71">
+    <row r="71" hidden="1">
       <c r="A71" t="s">
         <v>440</v>
       </c>
@@ -18941,7 +18941,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="72">
+    <row r="72" hidden="1">
       <c r="A72" t="s">
         <v>446</v>
       </c>
@@ -18994,7 +18994,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="73">
+    <row r="73" hidden="1">
       <c r="A73" t="s">
         <v>453</v>
       </c>
@@ -19047,7 +19047,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="74">
+    <row r="74" hidden="1">
       <c r="A74" t="s">
         <v>453</v>
       </c>
@@ -19100,7 +19100,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="75">
+    <row r="75" hidden="1">
       <c r="A75" t="s">
         <v>469</v>
       </c>
@@ -19153,7 +19153,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="76">
+    <row r="76" hidden="1">
       <c r="A76" t="s">
         <v>469</v>
       </c>
@@ -19206,7 +19206,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="77">
+    <row r="77" hidden="1">
       <c r="A77" t="s">
         <v>469</v>
       </c>
@@ -19259,7 +19259,7 @@
         <v>484</v>
       </c>
     </row>
-    <row r="78">
+    <row r="78" hidden="1">
       <c r="A78" t="s">
         <v>469</v>
       </c>
@@ -19312,7 +19312,7 @@
         <v>488</v>
       </c>
     </row>
-    <row r="79">
+    <row r="79" hidden="1">
       <c r="A79" t="s">
         <v>489</v>
       </c>
@@ -19365,7 +19365,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="80">
+    <row r="80" hidden="1">
       <c r="A80" t="s">
         <v>500</v>
       </c>
@@ -19418,7 +19418,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="81">
+    <row r="81" hidden="1">
       <c r="A81" t="s">
         <v>504</v>
       </c>
@@ -19471,7 +19471,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="82">
+    <row r="82" hidden="1">
       <c r="A82" t="s">
         <v>504</v>
       </c>
@@ -19524,7 +19524,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="83">
+    <row r="83" hidden="1">
       <c r="A83" t="s">
         <v>519</v>
       </c>
@@ -19577,7 +19577,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="84">
+    <row r="84" hidden="1">
       <c r="A84" t="s">
         <v>527</v>
       </c>
@@ -19630,7 +19630,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="85">
+    <row r="85" hidden="1">
       <c r="A85" t="s">
         <v>535</v>
       </c>
@@ -19683,7 +19683,7 @@
         <v>542</v>
       </c>
     </row>
-    <row r="86">
+    <row r="86" hidden="1">
       <c r="A86" t="s">
         <v>535</v>
       </c>
@@ -19736,7 +19736,7 @@
         <v>545</v>
       </c>
     </row>
-    <row r="87">
+    <row r="87" hidden="1">
       <c r="A87" t="s">
         <v>535</v>
       </c>
@@ -19789,7 +19789,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="88">
+    <row r="88" hidden="1">
       <c r="A88" t="s">
         <v>535</v>
       </c>
@@ -19842,7 +19842,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="89">
+    <row r="89" hidden="1">
       <c r="A89" t="s">
         <v>535</v>
       </c>
@@ -19895,7 +19895,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="90">
+    <row r="90" hidden="1">
       <c r="A90" t="s">
         <v>561</v>
       </c>
@@ -19948,7 +19948,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="91">
+    <row r="91" hidden="1">
       <c r="A91" t="s">
         <v>561</v>
       </c>
@@ -20001,7 +20001,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="92">
+    <row r="92" hidden="1">
       <c r="A92" t="s">
         <v>561</v>
       </c>
@@ -20054,7 +20054,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="93">
+    <row r="93" hidden="1">
       <c r="A93" t="s">
         <v>561</v>
       </c>
@@ -20107,7 +20107,7 @@
         <v>581</v>
       </c>
     </row>
-    <row r="94">
+    <row r="94" hidden="1">
       <c r="A94" t="s">
         <v>561</v>
       </c>
@@ -20160,7 +20160,7 @@
         <v>587</v>
       </c>
     </row>
-    <row r="95">
+    <row r="95" hidden="1">
       <c r="A95" t="s">
         <v>561</v>
       </c>
@@ -20213,7 +20213,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="96">
+    <row r="96" hidden="1">
       <c r="A96" t="s">
         <v>561</v>
       </c>
@@ -20266,7 +20266,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="97">
+    <row r="97" hidden="1">
       <c r="A97" t="s">
         <v>561</v>
       </c>
@@ -20319,7 +20319,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="98">
+    <row r="98" hidden="1">
       <c r="A98" t="s">
         <v>561</v>
       </c>
@@ -20372,7 +20372,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="99">
+    <row r="99" hidden="1">
       <c r="A99" t="s">
         <v>561</v>
       </c>
@@ -20425,7 +20425,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="100">
+    <row r="100" hidden="1">
       <c r="A100" t="s">
         <v>561</v>
       </c>
@@ -20478,7 +20478,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="101">
+    <row r="101" hidden="1">
       <c r="A101" t="s">
         <v>561</v>
       </c>
@@ -20531,7 +20531,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="102">
+    <row r="102" hidden="1">
       <c r="A102" t="s">
         <v>561</v>
       </c>
@@ -20584,7 +20584,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="103">
+    <row r="103" hidden="1">
       <c r="A103" t="s">
         <v>561</v>
       </c>
@@ -20637,7 +20637,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="104">
+    <row r="104" hidden="1">
       <c r="A104" t="s">
         <v>561</v>
       </c>
@@ -20690,7 +20690,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="105">
+    <row r="105" hidden="1">
       <c r="A105" t="s">
         <v>561</v>
       </c>
@@ -20743,7 +20743,7 @@
         <v>625</v>
       </c>
     </row>
-    <row r="106">
+    <row r="106" hidden="1">
       <c r="A106" t="s">
         <v>561</v>
       </c>
@@ -20796,7 +20796,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="107">
+    <row r="107" hidden="1">
       <c r="A107" t="s">
         <v>561</v>
       </c>
@@ -20849,7 +20849,7 @@
         <v>631</v>
       </c>
     </row>
-    <row r="108">
+    <row r="108" hidden="1">
       <c r="A108" t="s">
         <v>561</v>
       </c>
@@ -20902,7 +20902,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="109">
+    <row r="109" hidden="1">
       <c r="A109" t="s">
         <v>633</v>
       </c>
@@ -20955,7 +20955,7 @@
         <v>639</v>
       </c>
     </row>
-    <row r="110">
+    <row r="110" hidden="1">
       <c r="A110" t="s">
         <v>640</v>
       </c>
@@ -21008,7 +21008,7 @@
         <v>647</v>
       </c>
     </row>
-    <row r="111">
+    <row r="111" hidden="1">
       <c r="A111" t="s">
         <v>640</v>
       </c>
@@ -21061,7 +21061,7 @@
         <v>651</v>
       </c>
     </row>
-    <row r="112">
+    <row r="112" hidden="1">
       <c r="A112" t="s">
         <v>652</v>
       </c>
@@ -21114,7 +21114,7 @@
         <v>660</v>
       </c>
     </row>
-    <row r="113">
+    <row r="113" hidden="1">
       <c r="A113" t="s">
         <v>661</v>
       </c>
@@ -21167,7 +21167,7 @@
         <v>667</v>
       </c>
     </row>
-    <row r="114">
+    <row r="114" hidden="1">
       <c r="A114" t="s">
         <v>668</v>
       </c>
@@ -21220,7 +21220,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="115">
+    <row r="115" hidden="1">
       <c r="A115" t="s">
         <v>677</v>
       </c>
@@ -21273,7 +21273,7 @@
         <v>683</v>
       </c>
     </row>
-    <row r="116">
+    <row r="116" hidden="1">
       <c r="A116" t="s">
         <v>684</v>
       </c>
@@ -21326,7 +21326,7 @@
         <v>690</v>
       </c>
     </row>
-    <row r="117">
+    <row r="117" hidden="1">
       <c r="A117" t="s">
         <v>691</v>
       </c>
@@ -21379,7 +21379,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="118">
+    <row r="118" hidden="1">
       <c r="A118" t="s">
         <v>698</v>
       </c>
@@ -21432,7 +21432,7 @@
         <v>704</v>
       </c>
     </row>
-    <row r="119">
+    <row r="119" hidden="1">
       <c r="A119" t="s">
         <v>705</v>
       </c>
@@ -21485,7 +21485,7 @@
         <v>713</v>
       </c>
     </row>
-    <row r="120">
+    <row r="120" hidden="1">
       <c r="A120" t="s">
         <v>705</v>
       </c>
@@ -21538,7 +21538,7 @@
         <v>718</v>
       </c>
     </row>
-    <row r="121">
+    <row r="121" hidden="1">
       <c r="A121" t="s">
         <v>719</v>
       </c>
@@ -21591,7 +21591,7 @@
         <v>723</v>
       </c>
     </row>
-    <row r="122">
+    <row r="122" hidden="1">
       <c r="A122" t="s">
         <v>724</v>
       </c>
@@ -21644,7 +21644,7 @@
         <v>730</v>
       </c>
     </row>
-    <row r="123">
+    <row r="123" hidden="1">
       <c r="A123" t="s">
         <v>731</v>
       </c>
@@ -21697,7 +21697,7 @@
         <v>739</v>
       </c>
     </row>
-    <row r="124">
+    <row r="124" hidden="1">
       <c r="A124" t="s">
         <v>740</v>
       </c>
@@ -21750,7 +21750,7 @@
         <v>746</v>
       </c>
     </row>
-    <row r="125">
+    <row r="125" hidden="1">
       <c r="A125" t="s">
         <v>747</v>
       </c>
@@ -21803,7 +21803,7 @@
         <v>753</v>
       </c>
     </row>
-    <row r="126">
+    <row r="126" hidden="1">
       <c r="A126" t="s">
         <v>754</v>
       </c>
@@ -21856,7 +21856,7 @@
         <v>760</v>
       </c>
     </row>
-    <row r="127">
+    <row r="127" hidden="1">
       <c r="A127" t="s">
         <v>761</v>
       </c>
@@ -21909,7 +21909,7 @@
         <v>767</v>
       </c>
     </row>
-    <row r="128">
+    <row r="128" hidden="1">
       <c r="A128" t="s">
         <v>761</v>
       </c>
@@ -21962,7 +21962,7 @@
         <v>770</v>
       </c>
     </row>
-    <row r="129">
+    <row r="129" hidden="1">
       <c r="A129" t="s">
         <v>771</v>
       </c>
@@ -22015,7 +22015,7 @@
         <v>778</v>
       </c>
     </row>
-    <row r="130">
+    <row r="130" hidden="1">
       <c r="A130" t="s">
         <v>771</v>
       </c>
@@ -22068,7 +22068,7 @@
         <v>781</v>
       </c>
     </row>
-    <row r="131">
+    <row r="131" hidden="1">
       <c r="A131" t="s">
         <v>782</v>
       </c>
@@ -22121,7 +22121,7 @@
         <v>788</v>
       </c>
     </row>
-    <row r="132">
+    <row r="132" hidden="1">
       <c r="A132" t="s">
         <v>789</v>
       </c>
@@ -22171,7 +22171,7 @@
         <v>795</v>
       </c>
     </row>
-    <row r="133">
+    <row r="133" hidden="1">
       <c r="A133" t="s">
         <v>789</v>
       </c>
@@ -22224,7 +22224,7 @@
         <v>801</v>
       </c>
     </row>
-    <row r="134">
+    <row r="134" hidden="1">
       <c r="A134" t="s">
         <v>789</v>
       </c>
@@ -22277,7 +22277,7 @@
         <v>808</v>
       </c>
     </row>
-    <row r="135">
+    <row r="135" hidden="1">
       <c r="A135" t="s">
         <v>789</v>
       </c>
@@ -22330,7 +22330,7 @@
         <v>814</v>
       </c>
     </row>
-    <row r="136">
+    <row r="136" hidden="1">
       <c r="A136" t="s">
         <v>789</v>
       </c>
@@ -22383,7 +22383,7 @@
         <v>817</v>
       </c>
     </row>
-    <row r="137">
+    <row r="137" hidden="1">
       <c r="A137" t="s">
         <v>789</v>
       </c>
@@ -22436,7 +22436,7 @@
         <v>820</v>
       </c>
     </row>
-    <row r="138">
+    <row r="138" hidden="1">
       <c r="A138" t="s">
         <v>821</v>
       </c>
@@ -22489,7 +22489,7 @@
         <v>824</v>
       </c>
     </row>
-    <row r="139">
+    <row r="139" hidden="1">
       <c r="A139" t="s">
         <v>825</v>
       </c>
@@ -22542,7 +22542,7 @@
         <v>831</v>
       </c>
     </row>
-    <row r="140">
+    <row r="140" hidden="1">
       <c r="A140" t="s">
         <v>832</v>
       </c>
@@ -22595,7 +22595,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="141">
+    <row r="141" hidden="1">
       <c r="A141" t="s">
         <v>838</v>
       </c>
@@ -22633,7 +22633,7 @@
         <v>841</v>
       </c>
     </row>
-    <row r="142">
+    <row r="142" hidden="1">
       <c r="A142" t="s">
         <v>842</v>
       </c>
@@ -22686,7 +22686,7 @@
         <v>846</v>
       </c>
     </row>
-    <row r="143">
+    <row r="143" hidden="1">
       <c r="A143" t="s">
         <v>847</v>
       </c>
@@ -22739,7 +22739,7 @@
         <v>855</v>
       </c>
     </row>
-    <row r="144">
+    <row r="144" hidden="1">
       <c r="A144" t="s">
         <v>856</v>
       </c>
@@ -22792,7 +22792,7 @@
         <v>863</v>
       </c>
     </row>
-    <row r="145">
+    <row r="145" hidden="1">
       <c r="A145" t="s">
         <v>864</v>
       </c>
@@ -22845,7 +22845,7 @@
         <v>872</v>
       </c>
     </row>
-    <row r="146">
+    <row r="146" hidden="1">
       <c r="A146" t="s">
         <v>873</v>
       </c>
@@ -22898,7 +22898,7 @@
         <v>880</v>
       </c>
     </row>
-    <row r="147">
+    <row r="147" hidden="1">
       <c r="A147" t="s">
         <v>881</v>
       </c>
@@ -22951,7 +22951,7 @@
         <v>889</v>
       </c>
     </row>
-    <row r="148">
+    <row r="148" hidden="1">
       <c r="A148" t="s">
         <v>890</v>
       </c>
@@ -23004,7 +23004,7 @@
         <v>899</v>
       </c>
     </row>
-    <row r="149">
+    <row r="149" hidden="1">
       <c r="A149" t="s">
         <v>900</v>
       </c>
@@ -23057,7 +23057,7 @@
         <v>907</v>
       </c>
     </row>
-    <row r="150">
+    <row r="150" hidden="1">
       <c r="A150" t="s">
         <v>908</v>
       </c>
@@ -23095,7 +23095,7 @@
         <v>914</v>
       </c>
     </row>
-    <row r="151">
+    <row r="151" hidden="1">
       <c r="A151" t="s">
         <v>915</v>
       </c>
@@ -23148,7 +23148,7 @@
         <v>919</v>
       </c>
     </row>
-    <row r="152">
+    <row r="152" hidden="1">
       <c r="A152" t="s">
         <v>920</v>
       </c>
@@ -23201,7 +23201,7 @@
         <v>923</v>
       </c>
     </row>
-    <row r="153">
+    <row r="153" hidden="1">
       <c r="A153" t="s">
         <v>924</v>
       </c>
@@ -23254,7 +23254,7 @@
         <v>927</v>
       </c>
     </row>
-    <row r="154">
+    <row r="154" hidden="1">
       <c r="A154" t="s">
         <v>928</v>
       </c>
@@ -23307,7 +23307,7 @@
         <v>933</v>
       </c>
     </row>
-    <row r="155">
+    <row r="155" hidden="1">
       <c r="A155" t="s">
         <v>934</v>
       </c>
@@ -23360,7 +23360,7 @@
         <v>939</v>
       </c>
     </row>
-    <row r="156">
+    <row r="156" hidden="1">
       <c r="A156" t="s">
         <v>940</v>
       </c>
@@ -23413,7 +23413,7 @@
         <v>946</v>
       </c>
     </row>
-    <row r="157">
+    <row r="157" hidden="1">
       <c r="A157" t="s">
         <v>940</v>
       </c>
@@ -23466,7 +23466,7 @@
         <v>949</v>
       </c>
     </row>
-    <row r="158">
+    <row r="158" hidden="1">
       <c r="A158" t="s">
         <v>940</v>
       </c>
@@ -23519,7 +23519,7 @@
         <v>952</v>
       </c>
     </row>
-    <row r="159">
+    <row r="159" hidden="1">
       <c r="A159" t="s">
         <v>940</v>
       </c>
@@ -23572,7 +23572,7 @@
         <v>957</v>
       </c>
     </row>
-    <row r="160">
+    <row r="160" hidden="1">
       <c r="A160" t="s">
         <v>940</v>
       </c>
@@ -23625,7 +23625,7 @@
         <v>959</v>
       </c>
     </row>
-    <row r="161">
+    <row r="161" hidden="1">
       <c r="A161" t="s">
         <v>940</v>
       </c>
@@ -23678,7 +23678,7 @@
         <v>963</v>
       </c>
     </row>
-    <row r="162">
+    <row r="162" hidden="1">
       <c r="A162" t="s">
         <v>940</v>
       </c>
@@ -23731,7 +23731,7 @@
         <v>966</v>
       </c>
     </row>
-    <row r="163">
+    <row r="163" hidden="1">
       <c r="A163" t="s">
         <v>940</v>
       </c>
@@ -23784,7 +23784,7 @@
         <v>966</v>
       </c>
     </row>
-    <row r="164">
+    <row r="164" hidden="1">
       <c r="A164" t="s">
         <v>940</v>
       </c>
@@ -23837,7 +23837,7 @@
         <v>969</v>
       </c>
     </row>
-    <row r="165">
+    <row r="165" hidden="1">
       <c r="A165" t="s">
         <v>940</v>
       </c>
@@ -23890,7 +23890,7 @@
         <v>966</v>
       </c>
     </row>
-    <row r="166">
+    <row r="166" hidden="1">
       <c r="A166" t="s">
         <v>940</v>
       </c>
@@ -23943,7 +23943,7 @@
         <v>973</v>
       </c>
     </row>
-    <row r="167">
+    <row r="167" hidden="1">
       <c r="A167" t="s">
         <v>940</v>
       </c>
@@ -23996,7 +23996,7 @@
         <v>975</v>
       </c>
     </row>
-    <row r="168">
+    <row r="168" hidden="1">
       <c r="A168" t="s">
         <v>976</v>
       </c>
@@ -24049,7 +24049,7 @@
         <v>983</v>
       </c>
     </row>
-    <row r="169">
+    <row r="169" hidden="1">
       <c r="A169" t="s">
         <v>984</v>
       </c>
@@ -24102,7 +24102,7 @@
         <v>987</v>
       </c>
     </row>
-    <row r="170">
+    <row r="170" hidden="1">
       <c r="A170" t="s">
         <v>988</v>
       </c>
@@ -24155,7 +24155,7 @@
         <v>995</v>
       </c>
     </row>
-    <row r="171">
+    <row r="171" hidden="1">
       <c r="A171" t="s">
         <v>996</v>
       </c>
@@ -24193,7 +24193,7 @@
         <v>1001</v>
       </c>
     </row>
-    <row r="172">
+    <row r="172" hidden="1">
       <c r="A172" t="s">
         <v>1002</v>
       </c>
@@ -24246,7 +24246,7 @@
         <v>1008</v>
       </c>
     </row>
-    <row r="173">
+    <row r="173" hidden="1">
       <c r="A173" t="s">
         <v>1009</v>
       </c>
@@ -24299,7 +24299,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="174">
+    <row r="174" hidden="1">
       <c r="A174" t="s">
         <v>1009</v>
       </c>
@@ -24352,7 +24352,7 @@
         <v>1018</v>
       </c>
     </row>
-    <row r="175">
+    <row r="175" hidden="1">
       <c r="A175" t="s">
         <v>1009</v>
       </c>
@@ -24405,7 +24405,7 @@
         <v>1021</v>
       </c>
     </row>
-    <row r="176">
+    <row r="176" hidden="1">
       <c r="A176" t="s">
         <v>1009</v>
       </c>
@@ -24458,7 +24458,7 @@
         <v>1024</v>
       </c>
     </row>
-    <row r="177">
+    <row r="177" hidden="1">
       <c r="A177" t="s">
         <v>1009</v>
       </c>
@@ -24511,7 +24511,7 @@
         <v>1027</v>
       </c>
     </row>
-    <row r="178">
+    <row r="178" hidden="1">
       <c r="A178" t="s">
         <v>1009</v>
       </c>
@@ -24564,7 +24564,7 @@
         <v>1030</v>
       </c>
     </row>
-    <row r="179">
+    <row r="179" hidden="1">
       <c r="A179" t="s">
         <v>1009</v>
       </c>
@@ -24617,7 +24617,7 @@
         <v>1033</v>
       </c>
     </row>
-    <row r="180">
+    <row r="180" hidden="1">
       <c r="A180" t="s">
         <v>1034</v>
       </c>
@@ -24670,7 +24670,7 @@
         <v>1040</v>
       </c>
     </row>
-    <row r="181">
+    <row r="181" hidden="1">
       <c r="A181" t="s">
         <v>1041</v>
       </c>
@@ -24723,7 +24723,7 @@
         <v>1044</v>
       </c>
     </row>
-    <row r="182">
+    <row r="182" hidden="1">
       <c r="A182" t="s">
         <v>1045</v>
       </c>
@@ -24776,7 +24776,7 @@
         <v>1053</v>
       </c>
     </row>
-    <row r="183">
+    <row r="183" hidden="1">
       <c r="A183" t="s">
         <v>1045</v>
       </c>
@@ -24829,7 +24829,7 @@
         <v>1056</v>
       </c>
     </row>
-    <row r="184">
+    <row r="184" hidden="1">
       <c r="A184" t="s">
         <v>1057</v>
       </c>
@@ -24882,7 +24882,7 @@
         <v>1064</v>
       </c>
     </row>
-    <row r="185">
+    <row r="185" hidden="1">
       <c r="A185" t="s">
         <v>1057</v>
       </c>
@@ -24935,7 +24935,7 @@
         <v>1069</v>
       </c>
     </row>
-    <row r="186">
+    <row r="186" hidden="1">
       <c r="A186" t="s">
         <v>1070</v>
       </c>
@@ -24988,7 +24988,7 @@
         <v>1076</v>
       </c>
     </row>
-    <row r="187">
+    <row r="187" hidden="1">
       <c r="A187" t="s">
         <v>1077</v>
       </c>
@@ -25041,7 +25041,7 @@
         <v>1082</v>
       </c>
     </row>
-    <row r="188">
+    <row r="188" hidden="1">
       <c r="A188" t="s">
         <v>1077</v>
       </c>
@@ -25094,7 +25094,7 @@
         <v>1087</v>
       </c>
     </row>
-    <row r="189">
+    <row r="189" hidden="1">
       <c r="A189" t="s">
         <v>1077</v>
       </c>
@@ -25147,7 +25147,7 @@
         <v>1092</v>
       </c>
     </row>
-    <row r="190">
+    <row r="190" hidden="1">
       <c r="A190" t="s">
         <v>1077</v>
       </c>
@@ -25200,7 +25200,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="191">
+    <row r="191" hidden="1">
       <c r="A191" t="s">
         <v>1077</v>
       </c>
@@ -25253,7 +25253,7 @@
         <v>1102</v>
       </c>
     </row>
-    <row r="192">
+    <row r="192" hidden="1">
       <c r="A192" t="s">
         <v>1077</v>
       </c>
@@ -25306,7 +25306,7 @@
         <v>1107</v>
       </c>
     </row>
-    <row r="193">
+    <row r="193" hidden="1">
       <c r="A193" t="s">
         <v>1077</v>
       </c>
@@ -25359,7 +25359,7 @@
         <v>1112</v>
       </c>
     </row>
-    <row r="194">
+    <row r="194" hidden="1">
       <c r="A194" t="s">
         <v>1077</v>
       </c>
@@ -25412,7 +25412,7 @@
         <v>1117</v>
       </c>
     </row>
-    <row r="195">
+    <row r="195" hidden="1">
       <c r="A195" t="s">
         <v>1077</v>
       </c>
@@ -25465,7 +25465,7 @@
         <v>1122</v>
       </c>
     </row>
-    <row r="196">
+    <row r="196" hidden="1">
       <c r="A196" t="s">
         <v>1077</v>
       </c>
@@ -25518,7 +25518,7 @@
         <v>1127</v>
       </c>
     </row>
-    <row r="197">
+    <row r="197" hidden="1">
       <c r="A197" t="s">
         <v>1077</v>
       </c>
@@ -25571,7 +25571,7 @@
         <v>1129</v>
       </c>
     </row>
-    <row r="198">
+    <row r="198" hidden="1">
       <c r="A198" t="s">
         <v>1077</v>
       </c>
@@ -25624,7 +25624,7 @@
         <v>1134</v>
       </c>
     </row>
-    <row r="199">
+    <row r="199" hidden="1">
       <c r="A199" t="s">
         <v>1077</v>
       </c>
@@ -25677,7 +25677,7 @@
         <v>1140</v>
       </c>
     </row>
-    <row r="200">
+    <row r="200" hidden="1">
       <c r="A200" t="s">
         <v>1141</v>
       </c>
@@ -25730,7 +25730,7 @@
         <v>1148</v>
       </c>
     </row>
-    <row r="201">
+    <row r="201" hidden="1">
       <c r="A201" t="s">
         <v>1149</v>
       </c>
@@ -25783,7 +25783,7 @@
         <v>1154</v>
       </c>
     </row>
-    <row r="202">
+    <row r="202" hidden="1">
       <c r="A202" t="s">
         <v>1155</v>
       </c>
@@ -25836,7 +25836,7 @@
         <v>1159</v>
       </c>
     </row>
-    <row r="203">
+    <row r="203" hidden="1">
       <c r="A203" t="s">
         <v>1160</v>
       </c>
@@ -25889,7 +25889,7 @@
         <v>1165</v>
       </c>
     </row>
-    <row r="204">
+    <row r="204" hidden="1">
       <c r="A204" t="s">
         <v>1160</v>
       </c>
@@ -25942,7 +25942,7 @@
         <v>730</v>
       </c>
     </row>
-    <row r="205">
+    <row r="205" hidden="1">
       <c r="A205" t="s">
         <v>1167</v>
       </c>
@@ -25995,7 +25995,7 @@
         <v>1170</v>
       </c>
     </row>
-    <row r="206">
+    <row r="206" hidden="1">
       <c r="A206" t="s">
         <v>1171</v>
       </c>
@@ -26048,7 +26048,7 @@
         <v>1178</v>
       </c>
     </row>
-    <row r="207">
+    <row r="207" hidden="1">
       <c r="A207" t="s">
         <v>1179</v>
       </c>
@@ -26101,7 +26101,7 @@
         <v>1182</v>
       </c>
     </row>
-    <row r="208">
+    <row r="208" hidden="1">
       <c r="A208" t="s">
         <v>1183</v>
       </c>
@@ -26154,7 +26154,7 @@
         <v>1185</v>
       </c>
     </row>
-    <row r="209">
+    <row r="209" hidden="1">
       <c r="A209" t="s">
         <v>1183</v>
       </c>
@@ -26207,7 +26207,7 @@
         <v>1192</v>
       </c>
     </row>
-    <row r="210">
+    <row r="210" hidden="1">
       <c r="A210" t="s">
         <v>1183</v>
       </c>
@@ -26260,7 +26260,7 @@
         <v>1194</v>
       </c>
     </row>
-    <row r="211">
+    <row r="211" hidden="1">
       <c r="A211" t="s">
         <v>1195</v>
       </c>
@@ -26313,7 +26313,7 @@
         <v>1201</v>
       </c>
     </row>
-    <row r="212">
+    <row r="212" hidden="1">
       <c r="A212" t="s">
         <v>1202</v>
       </c>
@@ -26366,7 +26366,7 @@
         <v>1208</v>
       </c>
     </row>
-    <row r="213">
+    <row r="213" hidden="1">
       <c r="A213" t="s">
         <v>1202</v>
       </c>
@@ -26419,7 +26419,7 @@
         <v>1214</v>
       </c>
     </row>
-    <row r="214">
+    <row r="214" hidden="1">
       <c r="A214" t="s">
         <v>1202</v>
       </c>
@@ -26472,7 +26472,7 @@
         <v>1220</v>
       </c>
     </row>
-    <row r="215">
+    <row r="215" hidden="1">
       <c r="A215" t="s">
         <v>1202</v>
       </c>
@@ -26525,7 +26525,7 @@
         <v>1223</v>
       </c>
     </row>
-    <row r="216">
+    <row r="216" hidden="1">
       <c r="A216" t="s">
         <v>1224</v>
       </c>
@@ -26578,7 +26578,7 @@
         <v>1232</v>
       </c>
     </row>
-    <row r="217">
+    <row r="217" hidden="1">
       <c r="A217" t="s">
         <v>1233</v>
       </c>
@@ -26631,7 +26631,7 @@
         <v>1235</v>
       </c>
     </row>
-    <row r="218">
+    <row r="218" hidden="1">
       <c r="A218" t="s">
         <v>1236</v>
       </c>
@@ -26684,7 +26684,7 @@
         <v>1242</v>
       </c>
     </row>
-    <row r="219">
+    <row r="219" hidden="1">
       <c r="A219" t="s">
         <v>1236</v>
       </c>
@@ -26737,7 +26737,7 @@
         <v>1245</v>
       </c>
     </row>
-    <row r="220">
+    <row r="220" hidden="1">
       <c r="A220" t="s">
         <v>1246</v>
       </c>
@@ -26790,7 +26790,7 @@
         <v>1252</v>
       </c>
     </row>
-    <row r="221">
+    <row r="221" hidden="1">
       <c r="A221" t="s">
         <v>1253</v>
       </c>
@@ -26828,7 +26828,7 @@
         <v>1257</v>
       </c>
     </row>
-    <row r="222">
+    <row r="222" hidden="1">
       <c r="A222" t="s">
         <v>1258</v>
       </c>
@@ -26881,7 +26881,7 @@
         <v>1264</v>
       </c>
     </row>
-    <row r="223">
+    <row r="223" hidden="1">
       <c r="A223" t="s">
         <v>1265</v>
       </c>
@@ -26934,7 +26934,7 @@
         <v>1267</v>
       </c>
     </row>
-    <row r="224">
+    <row r="224" hidden="1">
       <c r="A224" t="s">
         <v>1268</v>
       </c>
@@ -26987,7 +26987,7 @@
         <v>1272</v>
       </c>
     </row>
-    <row r="225">
+    <row r="225" hidden="1">
       <c r="A225" t="s">
         <v>1273</v>
       </c>
@@ -27040,7 +27040,7 @@
         <v>1279</v>
       </c>
     </row>
-    <row r="226">
+    <row r="226" hidden="1">
       <c r="A226" t="s">
         <v>1273</v>
       </c>
@@ -27093,7 +27093,7 @@
         <v>1285</v>
       </c>
     </row>
-    <row r="227">
+    <row r="227" hidden="1">
       <c r="A227" t="s">
         <v>1273</v>
       </c>
@@ -27146,7 +27146,7 @@
         <v>1291</v>
       </c>
     </row>
-    <row r="228">
+    <row r="228" hidden="1">
       <c r="A228" t="s">
         <v>1273</v>
       </c>
@@ -27199,7 +27199,7 @@
         <v>1297</v>
       </c>
     </row>
-    <row r="229">
+    <row r="229" hidden="1">
       <c r="A229" t="s">
         <v>1273</v>
       </c>
@@ -27252,7 +27252,7 @@
         <v>1302</v>
       </c>
     </row>
-    <row r="230">
+    <row r="230" hidden="1">
       <c r="A230" t="s">
         <v>1273</v>
       </c>
@@ -27305,7 +27305,7 @@
         <v>1308</v>
       </c>
     </row>
-    <row r="231">
+    <row r="231" hidden="1">
       <c r="A231" t="s">
         <v>1273</v>
       </c>
@@ -27358,7 +27358,7 @@
         <v>1313</v>
       </c>
     </row>
-    <row r="232">
+    <row r="232" hidden="1">
       <c r="A232" t="s">
         <v>1273</v>
       </c>
@@ -27411,7 +27411,7 @@
         <v>1319</v>
       </c>
     </row>
-    <row r="233">
+    <row r="233" hidden="1">
       <c r="A233" t="s">
         <v>1273</v>
       </c>
@@ -27464,7 +27464,7 @@
         <v>1324</v>
       </c>
     </row>
-    <row r="234">
+    <row r="234" hidden="1">
       <c r="A234" t="s">
         <v>1273</v>
       </c>
@@ -27517,7 +27517,7 @@
         <v>1330</v>
       </c>
     </row>
-    <row r="235">
+    <row r="235" hidden="1">
       <c r="A235" t="s">
         <v>1273</v>
       </c>
@@ -27570,7 +27570,7 @@
         <v>1336</v>
       </c>
     </row>
-    <row r="236">
+    <row r="236" hidden="1">
       <c r="A236" t="s">
         <v>1273</v>
       </c>
@@ -27623,7 +27623,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="237">
+    <row r="237" hidden="1">
       <c r="A237" t="s">
         <v>1273</v>
       </c>
@@ -27676,7 +27676,7 @@
         <v>1348</v>
       </c>
     </row>
-    <row r="238">
+    <row r="238" hidden="1">
       <c r="A238" t="s">
         <v>1273</v>
       </c>
@@ -27729,7 +27729,7 @@
         <v>1354</v>
       </c>
     </row>
-    <row r="239">
+    <row r="239" hidden="1">
       <c r="A239" t="s">
         <v>1273</v>
       </c>
@@ -27782,7 +27782,7 @@
         <v>1356</v>
       </c>
     </row>
-    <row r="240">
+    <row r="240" hidden="1">
       <c r="A240" t="s">
         <v>1273</v>
       </c>
@@ -27835,7 +27835,7 @@
         <v>1359</v>
       </c>
     </row>
-    <row r="241">
+    <row r="241" hidden="1">
       <c r="A241" t="s">
         <v>1273</v>
       </c>
@@ -27888,7 +27888,7 @@
         <v>1366</v>
       </c>
     </row>
-    <row r="242">
+    <row r="242" hidden="1">
       <c r="A242" t="s">
         <v>1273</v>
       </c>
@@ -27941,7 +27941,7 @@
         <v>1372</v>
       </c>
     </row>
-    <row r="243">
+    <row r="243" hidden="1">
       <c r="A243" t="s">
         <v>1273</v>
       </c>
@@ -27994,7 +27994,7 @@
         <v>1378</v>
       </c>
     </row>
-    <row r="244">
+    <row r="244" hidden="1">
       <c r="A244" t="s">
         <v>1273</v>
       </c>
@@ -28047,7 +28047,7 @@
         <v>1385</v>
       </c>
     </row>
-    <row r="245">
+    <row r="245" hidden="1">
       <c r="A245" t="s">
         <v>1273</v>
       </c>
@@ -28100,7 +28100,7 @@
         <v>1391</v>
       </c>
     </row>
-    <row r="246">
+    <row r="246" hidden="1">
       <c r="A246" t="s">
         <v>1392</v>
       </c>
@@ -28135,7 +28135,7 @@
         <v>1394</v>
       </c>
     </row>
-    <row r="247">
+    <row r="247" hidden="1">
       <c r="A247" t="s">
         <v>1395</v>
       </c>
@@ -28188,7 +28188,7 @@
         <v>1398</v>
       </c>
     </row>
-    <row r="248">
+    <row r="248" hidden="1">
       <c r="A248" t="s">
         <v>1395</v>
       </c>
@@ -28241,7 +28241,7 @@
         <v>1403</v>
       </c>
     </row>
-    <row r="249">
+    <row r="249" hidden="1">
       <c r="A249" t="s">
         <v>1395</v>
       </c>
@@ -28294,7 +28294,7 @@
         <v>1406</v>
       </c>
     </row>
-    <row r="250">
+    <row r="250" hidden="1">
       <c r="A250" t="s">
         <v>1395</v>
       </c>
@@ -28347,7 +28347,7 @@
         <v>1409</v>
       </c>
     </row>
-    <row r="251">
+    <row r="251" hidden="1">
       <c r="A251" t="s">
         <v>1410</v>
       </c>
@@ -28400,7 +28400,7 @@
         <v>1414</v>
       </c>
     </row>
-    <row r="252">
+    <row r="252" hidden="1">
       <c r="A252" t="s">
         <v>1415</v>
       </c>
@@ -28453,7 +28453,7 @@
         <v>1420</v>
       </c>
     </row>
-    <row r="253">
+    <row r="253" hidden="1">
       <c r="A253" t="s">
         <v>1421</v>
       </c>
@@ -28506,7 +28506,7 @@
         <v>1424</v>
       </c>
     </row>
-    <row r="254">
+    <row r="254" hidden="1">
       <c r="A254" t="s">
         <v>1425</v>
       </c>
@@ -28559,7 +28559,7 @@
         <v>1432</v>
       </c>
     </row>
-    <row r="255">
+    <row r="255" hidden="1">
       <c r="A255" t="s">
         <v>1433</v>
       </c>
@@ -28612,7 +28612,7 @@
         <v>1440</v>
       </c>
     </row>
-    <row r="256">
+    <row r="256" hidden="1">
       <c r="A256" t="s">
         <v>1441</v>
       </c>
@@ -28665,7 +28665,7 @@
         <v>1447</v>
       </c>
     </row>
-    <row r="257">
+    <row r="257" hidden="1">
       <c r="A257" t="s">
         <v>1448</v>
       </c>
@@ -28718,7 +28718,7 @@
         <v>1453</v>
       </c>
     </row>
-    <row r="258">
+    <row r="258" hidden="1">
       <c r="A258" t="s">
         <v>1454</v>
       </c>
@@ -28771,7 +28771,7 @@
         <v>1461</v>
       </c>
     </row>
-    <row r="259">
+    <row r="259" hidden="1">
       <c r="A259" t="s">
         <v>1462</v>
       </c>
@@ -28824,7 +28824,7 @@
         <v>1464</v>
       </c>
     </row>
-    <row r="260">
+    <row r="260" hidden="1">
       <c r="A260" t="s">
         <v>1465</v>
       </c>
@@ -28877,7 +28877,7 @@
         <v>1472</v>
       </c>
     </row>
-    <row r="261">
+    <row r="261" hidden="1">
       <c r="A261" t="s">
         <v>1473</v>
       </c>
@@ -28930,7 +28930,7 @@
         <v>1479</v>
       </c>
     </row>
-    <row r="262">
+    <row r="262" hidden="1">
       <c r="A262" t="s">
         <v>1480</v>
       </c>
@@ -28983,7 +28983,7 @@
         <v>1487</v>
       </c>
     </row>
-    <row r="263">
+    <row r="263" hidden="1">
       <c r="A263" t="s">
         <v>1488</v>
       </c>
@@ -29036,7 +29036,7 @@
         <v>1495</v>
       </c>
     </row>
-    <row r="264">
+    <row r="264" hidden="1">
       <c r="A264" t="s">
         <v>1496</v>
       </c>
@@ -29089,7 +29089,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="265">
+    <row r="265" hidden="1">
       <c r="A265" t="s">
         <v>1496</v>
       </c>
@@ -29142,7 +29142,7 @@
         <v>1503</v>
       </c>
     </row>
-    <row r="266">
+    <row r="266" hidden="1">
       <c r="A266" t="s">
         <v>1496</v>
       </c>
@@ -29195,7 +29195,7 @@
         <v>1508</v>
       </c>
     </row>
-    <row r="267">
+    <row r="267" hidden="1">
       <c r="A267" t="s">
         <v>1496</v>
       </c>
@@ -29248,7 +29248,7 @@
         <v>1510</v>
       </c>
     </row>
-    <row r="268">
+    <row r="268" hidden="1">
       <c r="A268" t="s">
         <v>1511</v>
       </c>
@@ -29301,7 +29301,7 @@
         <v>1518</v>
       </c>
     </row>
-    <row r="269">
+    <row r="269" hidden="1">
       <c r="A269" t="s">
         <v>1519</v>
       </c>
@@ -29351,7 +29351,7 @@
         <v>1526</v>
       </c>
     </row>
-    <row r="270">
+    <row r="270" hidden="1">
       <c r="A270" t="s">
         <v>1527</v>
       </c>
@@ -29404,7 +29404,7 @@
         <v>1533</v>
       </c>
     </row>
-    <row r="271">
+    <row r="271" hidden="1">
       <c r="A271" t="s">
         <v>1534</v>
       </c>
@@ -29457,7 +29457,7 @@
         <v>1540</v>
       </c>
     </row>
-    <row r="272">
+    <row r="272" hidden="1">
       <c r="A272" t="s">
         <v>1534</v>
       </c>
@@ -29510,7 +29510,7 @@
         <v>1543</v>
       </c>
     </row>
-    <row r="273">
+    <row r="273" hidden="1">
       <c r="A273" t="s">
         <v>1534</v>
       </c>
@@ -29563,7 +29563,7 @@
         <v>1545</v>
       </c>
     </row>
-    <row r="274">
+    <row r="274" hidden="1">
       <c r="A274" t="s">
         <v>1546</v>
       </c>
@@ -29669,7 +29669,7 @@
         <v>1561</v>
       </c>
     </row>
-    <row r="276">
+    <row r="276" hidden="1">
       <c r="A276" t="s">
         <v>1553</v>
       </c>
@@ -29722,7 +29722,7 @@
         <v>1567</v>
       </c>
     </row>
-    <row r="277">
+    <row r="277" hidden="1">
       <c r="A277" t="s">
         <v>1553</v>
       </c>
@@ -29775,7 +29775,7 @@
         <v>1573</v>
       </c>
     </row>
-    <row r="278">
+    <row r="278" hidden="1">
       <c r="A278" t="s">
         <v>1553</v>
       </c>
@@ -29828,7 +29828,7 @@
         <v>1578</v>
       </c>
     </row>
-    <row r="279">
+    <row r="279" hidden="1">
       <c r="A279" t="s">
         <v>1553</v>
       </c>
@@ -29881,7 +29881,7 @@
         <v>1583</v>
       </c>
     </row>
-    <row r="280">
+    <row r="280" hidden="1">
       <c r="A280" t="s">
         <v>1553</v>
       </c>
@@ -29934,7 +29934,7 @@
         <v>1589</v>
       </c>
     </row>
-    <row r="281">
+    <row r="281" hidden="1">
       <c r="A281" t="s">
         <v>1553</v>
       </c>
@@ -29987,7 +29987,7 @@
         <v>1592</v>
       </c>
     </row>
-    <row r="282">
+    <row r="282" hidden="1">
       <c r="A282" t="s">
         <v>1553</v>
       </c>
@@ -30040,7 +30040,7 @@
         <v>1597</v>
       </c>
     </row>
-    <row r="283">
+    <row r="283" hidden="1">
       <c r="A283" t="s">
         <v>1553</v>
       </c>
@@ -30093,7 +30093,7 @@
         <v>1603</v>
       </c>
     </row>
-    <row r="284">
+    <row r="284" hidden="1">
       <c r="A284" t="s">
         <v>1553</v>
       </c>
@@ -30146,7 +30146,7 @@
         <v>1605</v>
       </c>
     </row>
-    <row r="285">
+    <row r="285" hidden="1">
       <c r="A285" t="s">
         <v>1606</v>
       </c>
@@ -30199,7 +30199,7 @@
         <v>1611</v>
       </c>
     </row>
-    <row r="286">
+    <row r="286" hidden="1">
       <c r="A286" t="s">
         <v>1612</v>
       </c>
@@ -30252,7 +30252,7 @@
         <v>1618</v>
       </c>
     </row>
-    <row r="287">
+    <row r="287" hidden="1">
       <c r="A287" t="s">
         <v>1612</v>
       </c>
@@ -30305,7 +30305,7 @@
         <v>1623</v>
       </c>
     </row>
-    <row r="288">
+    <row r="288" hidden="1">
       <c r="A288" t="s">
         <v>1612</v>
       </c>
@@ -30358,7 +30358,7 @@
         <v>1629</v>
       </c>
     </row>
-    <row r="289">
+    <row r="289" hidden="1">
       <c r="A289" t="s">
         <v>1612</v>
       </c>
@@ -30411,7 +30411,7 @@
         <v>1636</v>
       </c>
     </row>
-    <row r="290">
+    <row r="290" hidden="1">
       <c r="A290" t="s">
         <v>1612</v>
       </c>
@@ -30464,7 +30464,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="291">
+    <row r="291" hidden="1">
       <c r="A291" t="s">
         <v>1612</v>
       </c>
@@ -30517,7 +30517,7 @@
         <v>1648</v>
       </c>
     </row>
-    <row r="292">
+    <row r="292" hidden="1">
       <c r="A292" t="s">
         <v>1649</v>
       </c>
@@ -30570,7 +30570,7 @@
         <v>1655</v>
       </c>
     </row>
-    <row r="293">
+    <row r="293" hidden="1">
       <c r="A293" t="s">
         <v>1649</v>
       </c>
@@ -30623,7 +30623,7 @@
         <v>1661</v>
       </c>
     </row>
-    <row r="294">
+    <row r="294" hidden="1">
       <c r="A294" t="s">
         <v>1649</v>
       </c>
@@ -30676,7 +30676,7 @@
         <v>1664</v>
       </c>
     </row>
-    <row r="295">
+    <row r="295" hidden="1">
       <c r="A295" t="s">
         <v>1649</v>
       </c>
@@ -30729,7 +30729,7 @@
         <v>1669</v>
       </c>
     </row>
-    <row r="296">
+    <row r="296" hidden="1">
       <c r="A296" t="s">
         <v>1670</v>
       </c>
@@ -30782,7 +30782,7 @@
         <v>1673</v>
       </c>
     </row>
-    <row r="297">
+    <row r="297" hidden="1">
       <c r="A297" t="s">
         <v>1674</v>
       </c>
@@ -30835,7 +30835,7 @@
         <v>1682</v>
       </c>
     </row>
-    <row r="298">
+    <row r="298" hidden="1">
       <c r="A298" t="s">
         <v>1674</v>
       </c>
@@ -30888,7 +30888,7 @@
         <v>1686</v>
       </c>
     </row>
-    <row r="299">
+    <row r="299" hidden="1">
       <c r="A299" t="s">
         <v>1687</v>
       </c>
@@ -30941,7 +30941,7 @@
         <v>1689</v>
       </c>
     </row>
-    <row r="300">
+    <row r="300" hidden="1">
       <c r="A300" t="s">
         <v>1690</v>
       </c>
@@ -30994,7 +30994,7 @@
         <v>1696</v>
       </c>
     </row>
-    <row r="301">
+    <row r="301" hidden="1">
       <c r="A301" t="s">
         <v>1697</v>
       </c>
@@ -31047,7 +31047,7 @@
         <v>1703</v>
       </c>
     </row>
-    <row r="302">
+    <row r="302" hidden="1">
       <c r="A302" t="s">
         <v>1704</v>
       </c>
@@ -31100,7 +31100,7 @@
         <v>1709</v>
       </c>
     </row>
-    <row r="303">
+    <row r="303" hidden="1">
       <c r="A303" t="s">
         <v>1710</v>
       </c>
@@ -31153,7 +31153,7 @@
         <v>1716</v>
       </c>
     </row>
-    <row r="304">
+    <row r="304" hidden="1">
       <c r="A304" t="s">
         <v>1717</v>
       </c>
@@ -31206,7 +31206,7 @@
         <v>1724</v>
       </c>
     </row>
-    <row r="305">
+    <row r="305" hidden="1">
       <c r="A305" t="s">
         <v>1717</v>
       </c>
@@ -31259,7 +31259,7 @@
         <v>1727</v>
       </c>
     </row>
-    <row r="306">
+    <row r="306" hidden="1">
       <c r="A306" t="s">
         <v>1728</v>
       </c>
@@ -31312,7 +31312,7 @@
         <v>1734</v>
       </c>
     </row>
-    <row r="307">
+    <row r="307" hidden="1">
       <c r="A307" t="s">
         <v>1735</v>
       </c>
@@ -31365,7 +31365,7 @@
         <v>1739</v>
       </c>
     </row>
-    <row r="308">
+    <row r="308" hidden="1">
       <c r="A308" t="s">
         <v>1740</v>
       </c>
@@ -31418,7 +31418,7 @@
         <v>1746</v>
       </c>
     </row>
-    <row r="309">
+    <row r="309" hidden="1">
       <c r="A309" t="s">
         <v>1747</v>
       </c>
@@ -31468,7 +31468,7 @@
         <v>1752</v>
       </c>
     </row>
-    <row r="310">
+    <row r="310" hidden="1">
       <c r="A310" t="s">
         <v>1753</v>
       </c>
@@ -31521,7 +31521,7 @@
         <v>1758</v>
       </c>
     </row>
-    <row r="311">
+    <row r="311" hidden="1">
       <c r="A311" t="s">
         <v>1759</v>
       </c>
@@ -31574,7 +31574,7 @@
         <v>1764</v>
       </c>
     </row>
-    <row r="312">
+    <row r="312" hidden="1">
       <c r="A312" t="s">
         <v>1759</v>
       </c>
@@ -31627,7 +31627,7 @@
         <v>1768</v>
       </c>
     </row>
-    <row r="313">
+    <row r="313" hidden="1">
       <c r="A313" t="s">
         <v>1769</v>
       </c>
@@ -31680,7 +31680,7 @@
         <v>1775</v>
       </c>
     </row>
-    <row r="314">
+    <row r="314" hidden="1">
       <c r="A314" t="s">
         <v>1776</v>
       </c>
@@ -31733,7 +31733,7 @@
         <v>1782</v>
       </c>
     </row>
-    <row r="315">
+    <row r="315" hidden="1">
       <c r="A315" t="s">
         <v>1776</v>
       </c>
@@ -31786,7 +31786,7 @@
         <v>1788</v>
       </c>
     </row>
-    <row r="316">
+    <row r="316" hidden="1">
       <c r="A316" t="s">
         <v>1789</v>
       </c>
@@ -31839,7 +31839,7 @@
         <v>1795</v>
       </c>
     </row>
-    <row r="317">
+    <row r="317" hidden="1">
       <c r="A317" t="s">
         <v>1796</v>
       </c>
@@ -31892,7 +31892,7 @@
         <v>1802</v>
       </c>
     </row>
-    <row r="318">
+    <row r="318" hidden="1">
       <c r="A318" t="s">
         <v>1803</v>
       </c>
@@ -31945,7 +31945,7 @@
         <v>1802</v>
       </c>
     </row>
-    <row r="319">
+    <row r="319" hidden="1">
       <c r="A319" t="s">
         <v>1805</v>
       </c>
@@ -31998,7 +31998,7 @@
         <v>1811</v>
       </c>
     </row>
-    <row r="320">
+    <row r="320" hidden="1">
       <c r="A320" t="s">
         <v>1812</v>
       </c>
@@ -32049,7 +32049,13 @@
       <c r="Q324" s="3"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q320"/>
+  <autoFilter ref="A1:Q320">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="SUZANO - ACAILANDIA"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157500000008" bottom="0.78740157500000008" header="0.31496062000000014" footer="0.31496062000000014"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
@@ -34975,7 +34981,7 @@
         <xsd:restriction base="dms:Unknown"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="_Flow_SignoffStatus" ma:index="21" nillable="true" ma:displayName="Status de liberação" ma:internalName="_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x0024_Resources_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x003a_core_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x002c_Signoff_Status">
+    <xsd:element name="_Flow_SignoffStatus" ma:index="21" nillable="true" ma:displayName="Status de liberação" ma:internalName="_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x0024_Resources_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x003a_core_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x002c_Signoff_Status">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>

</xml_diff>

<commit_message>
Add filial + Plus Code
</commit_message>
<xml_diff>
--- a/Mapa - Zelar.xlsx
+++ b/Mapa - Zelar.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Mapa" sheetId="1" state="visible" r:id="rId5"/>
@@ -5508,7 +5508,7 @@
     <t>Contagem</t>
   </si>
   <si>
-    <t xml:space="preserve">Unidas Seminovos, Av. Maria da Glória Rocha, 315 - Centro, Contagem - MG, 32010-375</t>
+    <t xml:space="preserve">3WGF+474 - Parque Industrial, Contagem - MG</t>
   </si>
   <si>
     <t xml:space="preserve">Edmar Marques</t>
@@ -5523,7 +5523,7 @@
     <t>Mauá</t>
   </si>
   <si>
-    <t xml:space="preserve">Unidas Seminovos, Av. Papa João XXIII, 3107 - Parque Sao Vicente, Mauá - SP, 09370-800</t>
+    <t xml:space="preserve">8G4G+4V, Mauá - SP</t>
   </si>
   <si>
     <t xml:space="preserve">Marcelo Nabor</t>
@@ -5538,7 +5538,7 @@
     <t>Curitiba</t>
   </si>
   <si>
-    <t xml:space="preserve">Unidas Seminovos Atacado, R. João Bettega, 5133b - Portão, Curitiba - PR, 81350-570</t>
+    <t xml:space="preserve">FMWC+GW, Curitiba - PR</t>
   </si>
   <si>
     <t xml:space="preserve">Marcelo Marques</t>
@@ -5553,7 +5553,7 @@
     <t>Sertãozinho</t>
   </si>
   <si>
-    <t xml:space="preserve">Av. Marginal Antônio Aragão, 1311 - Sertãozinho, SP, 14171-700</t>
+    <t xml:space="preserve">R2QC+4X - Cruz das Posses, Sertãozinho - SP</t>
   </si>
   <si>
     <t xml:space="preserve">João Corbo</t>
@@ -35207,7 +35207,7 @@
         <xsd:restriction base="dms:Unknown"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="_Flow_SignoffStatus" ma:index="21" nillable="true" ma:displayName="Status de liberação" ma:internalName="_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x0024_Resources_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x003a_core_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x002c_Signoff_Status">
+    <xsd:element name="_Flow_SignoffStatus" ma:index="21" nillable="true" ma:displayName="Status de liberação" ma:internalName="_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x0024_Resources_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x003a_core_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x005F_x002c_Signoff_Status">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>

</xml_diff>

<commit_message>
Add atualizaçao de viagem
</commit_message>
<xml_diff>
--- a/Mapa - Zelar.xlsx
+++ b/Mapa - Zelar.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aguinir.junior\Desktop\Gestão\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF27428C-A34D-430F-990E-E4779FC0EB9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18D31811-AD25-46F4-A38C-FF05B2324356}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
   </definedNames>
   <calcPr calcId="0"/>
   <pivotCaches>
-    <pivotCache cacheId="1" r:id="rId4"/>
+    <pivotCache cacheId="0" r:id="rId4"/>
   </pivotCaches>
 </workbook>
 </file>
@@ -5747,7 +5747,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -5759,6 +5759,7 @@
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -13002,7 +13003,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0100-000000000000}" name="Tabela dinâmica1" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0100-000000000000}" name="Tabela dinâmica1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A5:B348" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="3" colPageCount="1"/>
   <pivotFields count="17">
     <pivotField showAll="0" sortType="descending">
@@ -15168,7 +15169,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>43</v>
       </c>
@@ -15592,7 +15593,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>1160</v>
       </c>
@@ -18984,7 +18985,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="76" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>1750</v>
       </c>
@@ -19140,7 +19141,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="79" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>706</v>
       </c>
@@ -20412,7 +20413,7 @@
         <v>616</v>
       </c>
     </row>
-    <row r="103" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>563</v>
       </c>
@@ -20422,8 +20423,8 @@
       <c r="C103" t="s">
         <v>55</v>
       </c>
-      <c r="D103" t="s">
-        <v>45</v>
+      <c r="D103" s="7" t="s">
+        <v>250</v>
       </c>
       <c r="E103" t="s">
         <v>114</v>
@@ -21260,7 +21261,7 @@
         <v>705</v>
       </c>
     </row>
-    <row r="119" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>911</v>
       </c>
@@ -21298,7 +21299,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="120" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>470</v>
       </c>
@@ -22408,7 +22409,7 @@
         <v>839</v>
       </c>
     </row>
-    <row r="141" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>849</v>
       </c>
@@ -22514,7 +22515,7 @@
         <v>848</v>
       </c>
     </row>
-    <row r="143" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>1172</v>
       </c>
@@ -22885,7 +22886,7 @@
         <v>910</v>
       </c>
     </row>
-    <row r="150" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>1258</v>
       </c>
@@ -23082,7 +23083,7 @@
         <v>930</v>
       </c>
     </row>
-    <row r="154" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>1557</v>
       </c>
@@ -23135,7 +23136,7 @@
         <v>1595</v>
       </c>
     </row>
-    <row r="155" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>1673</v>
       </c>
@@ -23983,7 +23984,7 @@
         <v>999</v>
       </c>
     </row>
-    <row r="171" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>1738</v>
       </c>
@@ -25626,7 +25627,7 @@
         <v>1159</v>
       </c>
     </row>
-    <row r="202" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
         <v>1762</v>
       </c>
@@ -25785,7 +25786,7 @@
         <v>732</v>
       </c>
     </row>
-    <row r="205" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A205" t="s">
         <v>490</v>
       </c>
@@ -26633,7 +26634,7 @@
         <v>1257</v>
       </c>
     </row>
-    <row r="221" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A221" t="s">
         <v>937</v>
       </c>
@@ -29159,7 +29160,7 @@
         <v>1522</v>
       </c>
     </row>
-    <row r="269" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A269" t="s">
         <v>1523</v>
       </c>
@@ -29792,7 +29793,7 @@
         <v>1592</v>
       </c>
     </row>
-    <row r="281" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A281" t="s">
         <v>931</v>
       </c>
@@ -30375,7 +30376,7 @@
         <v>1651</v>
       </c>
     </row>
-    <row r="292" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A292" t="s">
         <v>1762</v>
       </c>
@@ -30587,7 +30588,7 @@
         <v>1672</v>
       </c>
     </row>
-    <row r="296" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A296" t="s">
         <v>1808</v>
       </c>
@@ -30640,7 +30641,7 @@
         <v>1814</v>
       </c>
     </row>
-    <row r="297" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A297" t="s">
         <v>706</v>
       </c>
@@ -30693,7 +30694,7 @@
         <v>720</v>
       </c>
     </row>
-    <row r="298" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A298" t="s">
         <v>111</v>
       </c>
@@ -31161,7 +31162,7 @@
         <v>1737</v>
       </c>
     </row>
-    <row r="307" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A307" t="s">
         <v>840</v>
       </c>
@@ -31252,7 +31253,7 @@
         <v>1749</v>
       </c>
     </row>
-    <row r="309" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="309" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A309" t="s">
         <v>1000</v>
       </c>
@@ -31343,7 +31344,7 @@
         <v>1761</v>
       </c>
     </row>
-    <row r="311" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="311" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A311" t="s">
         <v>1652</v>
       </c>
@@ -31396,7 +31397,7 @@
         <v>1658</v>
       </c>
     </row>
-    <row r="312" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="312" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A312" t="s">
         <v>1806</v>
       </c>
@@ -31714,7 +31715,7 @@
         <v>1805</v>
       </c>
     </row>
-    <row r="318" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="318" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A318" t="s">
         <v>1677</v>
       </c>
@@ -31767,7 +31768,7 @@
         <v>1685</v>
       </c>
     </row>
-    <row r="319" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="319" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A319" t="s">
         <v>1677</v>
       </c>
@@ -31869,23 +31870,11 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:Q320" xr:uid="{00000000-0009-0000-0000-000000000000}">
-    <filterColumn colId="2">
+    <filterColumn colId="1">
       <filters>
-        <filter val="ABRIL/25"/>
-        <filter val="AGOSTO/25"/>
-        <filter val="DEZEMBRO/25"/>
-        <filter val="FEVEREIRO/25"/>
-        <filter val="JANEIRO/25"/>
-        <filter val="JULHO/25"/>
-        <filter val="JUNHO/25"/>
-        <filter val="MAIO/25"/>
-        <filter val="NOVEMBRO/25"/>
-        <filter val="SETEMBRO/25"/>
+        <filter val="CITROSUCO - FAZENDA SAO CARLOS"/>
       </filters>
     </filterColumn>
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:Q319">
-      <sortCondition ref="C1:C320"/>
-    </sortState>
   </autoFilter>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157500000008" bottom="0.78740157500000008" header="0.31496062000000014" footer="0.31496062000000014"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -34821,15 +34810,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f71fe8f7-59e0-4170-8335-c26c48765730">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <_Flow_SignoffStatus xmlns="f71fe8f7-59e0-4170-8335-c26c48765730" xsi:nil="true"/>
-    <TaxCatchAll xmlns="ae1994d5-d842-4ca1-8495-71b46b36cfda" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -35044,22 +35030,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f71fe8f7-59e0-4170-8335-c26c48765730">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <_Flow_SignoffStatus xmlns="f71fe8f7-59e0-4170-8335-c26c48765730" xsi:nil="true"/>
+    <TaxCatchAll xmlns="ae1994d5-d842-4ca1-8495-71b46b36cfda" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E72E0B9D-311B-47AA-B002-82B0732EB526}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7608F113-E40D-4867-9E74-D7267DA6B4B0}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="f71fe8f7-59e0-4170-8335-c26c48765730"/>
-    <ds:schemaRef ds:uri="ae1994d5-d842-4ca1-8495-71b46b36cfda"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema-instance"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -35085,9 +35070,13 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7608F113-E40D-4867-9E74-D7267DA6B4B0}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E72E0B9D-311B-47AA-B002-82B0732EB526}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="f71fe8f7-59e0-4170-8335-c26c48765730"/>
+    <ds:schemaRef ds:uri="ae1994d5-d842-4ca1-8495-71b46b36cfda"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema-instance"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>